<commit_message>
two force with micro perturb full results
</commit_message>
<xml_diff>
--- a/testdata.xlsx
+++ b/testdata.xlsx
@@ -58,7 +58,7 @@
   <cols>
     <col min="1" max="1" width="12.7109375" customWidth="true"/>
     <col min="2" max="2" width="13.7109375" customWidth="true"/>
-    <col min="3" max="3" width="12.7109375" customWidth="true"/>
+    <col min="3" max="3" width="11.7109375" customWidth="true"/>
     <col min="4" max="4" width="11.7109375" customWidth="true"/>
     <col min="5" max="5" width="12.7109375" customWidth="true"/>
     <col min="6" max="6" width="13.7109375" customWidth="true"/>
@@ -69,437 +69,437 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0">
-        <v>0.76363365135228745</v>
+        <v>0.36812589768930226</v>
       </c>
       <c r="B1" s="0">
-        <v>0.08888519016512933</v>
+        <v>0.15632348649605163</v>
       </c>
       <c r="C1" s="0">
-        <v>1.5915908584895087</v>
+        <v>1.529531460180177</v>
       </c>
       <c r="D1" s="0">
         <v>1.5707963267948966</v>
       </c>
       <c r="E1" s="0">
-        <v>0.43678569903044911</v>
+        <v>0.30024142250950914</v>
       </c>
       <c r="F1" s="0">
-        <v>0.024746642498929054</v>
+        <v>0.03101431493391834</v>
       </c>
       <c r="G1" s="0">
-        <v>4.0522915968346922</v>
+        <v>3.1262104863074311</v>
       </c>
       <c r="H1" s="0">
         <v>1.5707963267948966</v>
       </c>
       <c r="I1" s="0">
-        <v>1.0218740945602944e-08</v>
+        <v>1.3240492512382839e-06</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="0">
-        <v>0.2361928483768298</v>
+        <v>0.56004930068563363</v>
       </c>
       <c r="B2" s="0">
-        <v>0.12963296786042683</v>
+        <v>0.16686693714739556</v>
       </c>
       <c r="C2" s="0">
-        <v>1.6532551903303669</v>
+        <v>1.534819317952397</v>
       </c>
       <c r="D2" s="0">
         <v>1.5707963267948966</v>
       </c>
       <c r="E2" s="0">
-        <v>0.42307346571120047</v>
+        <v>0.68274928290561365</v>
       </c>
       <c r="F2" s="0">
-        <v>0.020000017626560177</v>
+        <v>0.094720719090467115</v>
       </c>
       <c r="G2" s="0">
-        <v>4.7519267340730167</v>
+        <v>4.6774162642617716</v>
       </c>
       <c r="H2" s="0">
         <v>1.5707963267948966</v>
       </c>
       <c r="I2" s="0">
-        <v>1.9019607825814942e-07</v>
+        <v>7.6862678292148174e-06</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0">
-        <v>0.75817542182106845</v>
+        <v>0.85920177522492991</v>
       </c>
       <c r="B3" s="0">
-        <v>0.18070210151059904</v>
+        <v>0.18519334189436665</v>
       </c>
       <c r="C3" s="0">
-        <v>1.6018341710038033</v>
+        <v>1.6012035230502721</v>
       </c>
       <c r="D3" s="0">
         <v>1.5707963267948966</v>
       </c>
       <c r="E3" s="0">
-        <v>0.30463689776690051</v>
+        <v>0.47344361257026446</v>
       </c>
       <c r="F3" s="0">
-        <v>0.032462969578982204</v>
+        <v>0.10687620803731127</v>
       </c>
       <c r="G3" s="0">
-        <v>4.779461427088977</v>
+        <v>4.8430913984623603</v>
       </c>
       <c r="H3" s="0">
         <v>1.5707963267948966</v>
       </c>
       <c r="I3" s="0">
-        <v>2.192318654833206e-07</v>
+        <v>1.3311327359854187e-05</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0">
-        <v>0.52721599036919065</v>
+        <v>0.29978582893680189</v>
       </c>
       <c r="B4" s="0">
-        <v>0.13064266340979669</v>
+        <v>0.19980744544364126</v>
       </c>
       <c r="C4" s="0">
-        <v>1.5692194584815133</v>
+        <v>1.4734900722218307</v>
       </c>
       <c r="D4" s="0">
         <v>1.5707963267948966</v>
       </c>
       <c r="E4" s="0">
-        <v>0.77627959066504493</v>
+        <v>0.72588706707290052</v>
       </c>
       <c r="F4" s="0">
-        <v>0.04483867146613775</v>
+        <v>0.049748908514736456</v>
       </c>
       <c r="G4" s="0">
-        <v>3.6594988321543296</v>
+        <v>3.4079606035096717</v>
       </c>
       <c r="H4" s="0">
         <v>1.5707963267948966</v>
       </c>
       <c r="I4" s="0">
-        <v>6.96360561720752e-08</v>
+        <v>3.4862002203800943e-06</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0">
-        <v>0.60713301008119613</v>
+        <v>0.6806331994574889</v>
       </c>
       <c r="B5" s="0">
-        <v>0.090858055647504404</v>
+        <v>0.086026430432652817</v>
       </c>
       <c r="C5" s="0">
-        <v>2.9813250275329457</v>
+        <v>2.9409907946849319</v>
       </c>
       <c r="D5" s="0">
         <v>1.5707963267948966</v>
       </c>
       <c r="E5" s="0">
-        <v>0.66459208617919552</v>
+        <v>0.67901010121903682</v>
       </c>
       <c r="F5" s="0">
-        <v>0.086605784603893468</v>
+        <v>0.080471232759914829</v>
       </c>
       <c r="G5" s="0">
-        <v>4.2368231284953302</v>
+        <v>4.4003431901341186</v>
       </c>
       <c r="H5" s="0">
         <v>1.5707963267948966</v>
       </c>
       <c r="I5" s="0">
-        <v>2.7453203073212905e-06</v>
+        <v>8.1464082771986257e-06</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="0">
-        <v>0.8144252781731437</v>
+        <v>0.77393892308662438</v>
       </c>
       <c r="B6" s="0">
-        <v>0.096125258969866748</v>
+        <v>0.082857599157317233</v>
       </c>
       <c r="C6" s="0">
-        <v>2.8815087289782082</v>
+        <v>3.1045395242461655</v>
       </c>
       <c r="D6" s="0">
         <v>1.5707963267948966</v>
       </c>
       <c r="E6" s="0">
-        <v>0.52750015746723689</v>
+        <v>0.43045698478271283</v>
       </c>
       <c r="F6" s="0">
-        <v>0.074228373720110985</v>
+        <v>0.048545751751218176</v>
       </c>
       <c r="G6" s="0">
-        <v>4.1023158331038303</v>
+        <v>3.8935493864284476</v>
       </c>
       <c r="H6" s="0">
         <v>1.5707963267948966</v>
       </c>
       <c r="I6" s="0">
-        <v>3.7668415371455878e-07</v>
+        <v>1.9358100401641475e-05</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="0">
-        <v>0.64637441469415347</v>
+        <v>0.24090802440847459</v>
       </c>
       <c r="B7" s="0">
-        <v>0.12953535920944981</v>
+        <v>0.15326383679369923</v>
       </c>
       <c r="C7" s="0">
-        <v>2.8837153646999623</v>
+        <v>2.867759016008355</v>
       </c>
       <c r="D7" s="0">
         <v>1.5707963267948966</v>
       </c>
       <c r="E7" s="0">
-        <v>0.68389247067324233</v>
+        <v>0.92856669670630876</v>
       </c>
       <c r="F7" s="0">
-        <v>0.1043476293615514</v>
+        <v>0.085631391217949729</v>
       </c>
       <c r="G7" s="0">
-        <v>4.0916041799748522</v>
+        <v>3.6422948784847131</v>
       </c>
       <c r="H7" s="0">
         <v>1.5707963267948966</v>
       </c>
       <c r="I7" s="0">
-        <v>9.2540084858739116e-07</v>
+        <v>1.706338825363683e-05</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="0">
-        <v>0.77057969060101694</v>
+        <v>0.69162729491676089</v>
       </c>
       <c r="B8" s="0">
-        <v>0.13106213675642675</v>
+        <v>0.11092201197710488</v>
       </c>
       <c r="C8" s="0">
-        <v>2.8258416527406154</v>
+        <v>3.0127857942366614</v>
       </c>
       <c r="D8" s="0">
         <v>1.5707963267948966</v>
       </c>
       <c r="E8" s="0">
-        <v>0.63701334027023304</v>
+        <v>0.73867832090078001</v>
       </c>
       <c r="F8" s="0">
-        <v>0.099807208834126471</v>
+        <v>0.065091239748481869</v>
       </c>
       <c r="G8" s="0">
-        <v>4.1514962125184747</v>
+        <v>3.8151842033432355</v>
       </c>
       <c r="H8" s="0">
         <v>1.5707963267948966</v>
       </c>
       <c r="I8" s="0">
-        <v>9.7908619354922661e-07</v>
+        <v>4.2574098699885561e-05</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="0">
-        <v>0.26678114285968224</v>
+        <v>0.44227332682612736</v>
       </c>
       <c r="B9" s="0">
-        <v>0.18110205090970105</v>
+        <v>0.18485320333525496</v>
       </c>
       <c r="C9" s="0">
-        <v>2.4156391455236372</v>
+        <v>3.1601558205378004</v>
       </c>
       <c r="D9" s="0">
         <v>1.5707963267948966</v>
       </c>
       <c r="E9" s="0">
-        <v>0.5941161585705077</v>
+        <v>0.32131769996080994</v>
       </c>
       <c r="F9" s="0">
-        <v>0.093832982205083446</v>
+        <v>0.027491822674676578</v>
       </c>
       <c r="G9" s="0">
-        <v>3.9005298078518709</v>
+        <v>4.0307143013635649</v>
       </c>
       <c r="H9" s="0">
         <v>1.5707963267948966</v>
       </c>
       <c r="I9" s="0">
-        <v>6.1997032788828846e-07</v>
+        <v>3.7671144603751207e-06</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="0">
-        <v>0.97831711335596638</v>
+        <v>0.35705684567240348</v>
       </c>
       <c r="B10" s="0">
-        <v>0.15277152791140047</v>
+        <v>0.16128237383631006</v>
       </c>
       <c r="C10" s="0">
-        <v>3.0942799368390244</v>
+        <v>1.5220114176391086</v>
       </c>
       <c r="D10" s="0">
         <v>1.5707963267948966</v>
       </c>
       <c r="E10" s="0">
-        <v>0.60983392468265252</v>
+        <v>0.30503872897248818</v>
       </c>
       <c r="F10" s="0">
-        <v>0.060676688669076488</v>
+        <v>0.031805446057841115</v>
       </c>
       <c r="G10" s="0">
-        <v>4.1349589044002881</v>
+        <v>3.1029548174512036</v>
       </c>
       <c r="H10" s="0">
         <v>1.5707963267948966</v>
       </c>
       <c r="I10" s="0">
-        <v>1.4352086796852891e-06</v>
+        <v>2.0123723052764442e-06</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="0">
-        <v>0.17620896176457868</v>
+        <v>0.38361274929049743</v>
       </c>
       <c r="B11" s="0">
-        <v>0.099286257032007066</v>
+        <v>0.11941426198311951</v>
       </c>
       <c r="C11" s="0">
-        <v>0.12186637325268596</v>
+        <v>4.6791184330747715</v>
       </c>
       <c r="D11" s="0">
         <v>1.5707963267948966</v>
       </c>
       <c r="E11" s="0">
-        <v>0.65619757764419362</v>
+        <v>0.16441798445049088</v>
       </c>
       <c r="F11" s="0">
-        <v>0.088113330033240705</v>
+        <v>0.023999915201576027</v>
       </c>
       <c r="G11" s="0">
-        <v>4.3571793173094253</v>
+        <v>4.3756608637894479</v>
       </c>
       <c r="H11" s="0">
         <v>1.5707963267948966</v>
       </c>
       <c r="I11" s="0">
-        <v>8.7905820271715823e-08</v>
+        <v>9.9352468816000884e-07</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="0">
-        <v>0.95728856181666944</v>
+        <v>0.57884488557674163</v>
       </c>
       <c r="B12" s="0">
-        <v>0.11629478017871611</v>
+        <v>0.1342860126946413</v>
       </c>
       <c r="C12" s="0">
-        <v>4.6704620216669444</v>
+        <v>4.8180208803924716</v>
       </c>
       <c r="D12" s="0">
         <v>1.5707963267948966</v>
       </c>
       <c r="E12" s="0">
-        <v>0.66378324995961235</v>
+        <v>0.9055598607527191</v>
       </c>
       <c r="F12" s="0">
-        <v>0.020010429330519604</v>
+        <v>0.027514195310973343</v>
       </c>
       <c r="G12" s="0">
-        <v>3.0768212349740671</v>
+        <v>3.6914931016924668</v>
       </c>
       <c r="H12" s="0">
         <v>1.5707963267948966</v>
       </c>
       <c r="I12" s="0">
-        <v>4.2614175506698193e-07</v>
+        <v>3.758143940003182e-05</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="0">
-        <v>0.69971262479204777</v>
+        <v>0.36903295678703757</v>
       </c>
       <c r="B13" s="0">
-        <v>0.11556320577332801</v>
+        <v>0.19896050699611009</v>
       </c>
       <c r="C13" s="0">
-        <v>4.415148212454814</v>
+        <v>4.8428322746841319</v>
       </c>
       <c r="D13" s="0">
         <v>1.5707963267948966</v>
       </c>
       <c r="E13" s="0">
-        <v>0.40924275139356486</v>
+        <v>0.52304822935629181</v>
       </c>
       <c r="F13" s="0">
-        <v>0.020993314529002112</v>
+        <v>0.072909479066983626</v>
       </c>
       <c r="G13" s="0">
-        <v>2.3753136829666475</v>
+        <v>3.166876271307697</v>
       </c>
       <c r="H13" s="0">
         <v>1.5707963267948966</v>
       </c>
       <c r="I13" s="0">
-        <v>3.8088550880511999e-07</v>
+        <v>3.9443999910919594e-06</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="0">
-        <v>0.62762904706019684</v>
+        <v>0.50248823188162883</v>
       </c>
       <c r="B14" s="0">
-        <v>0.15592001226964788</v>
+        <v>0.19691519977181102</v>
       </c>
       <c r="C14" s="0">
-        <v>4.6658380803727662</v>
+        <v>4.6703707719310534</v>
       </c>
       <c r="D14" s="0">
         <v>1.5707963267948966</v>
       </c>
       <c r="E14" s="0">
-        <v>0.44377945999398916</v>
+        <v>0.65787117500335124</v>
       </c>
       <c r="F14" s="0">
-        <v>0.020084377410258255</v>
+        <v>0.020000000000022205</v>
       </c>
       <c r="G14" s="0">
-        <v>4.674487308102333</v>
+        <v>4.4666205933662537</v>
       </c>
       <c r="H14" s="0">
         <v>1.5707963267948966</v>
       </c>
       <c r="I14" s="0">
-        <v>2.9722812632829164e-06</v>
+        <v>2.3669180565077491e-05</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="0">
-        <v>0.80051743502710881</v>
+        <v>0.3610082897573525</v>
       </c>
       <c r="B15" s="0">
-        <v>0.19812384042746445</v>
+        <v>0.16094511301474176</v>
       </c>
       <c r="C15" s="0">
-        <v>4.742777937040966</v>
+        <v>1.5261251170999763</v>
       </c>
       <c r="D15" s="0">
         <v>1.5707963267948966</v>
       </c>
       <c r="E15" s="0">
-        <v>0.34005316031621635</v>
+        <v>0.30531802559027493</v>
       </c>
       <c r="F15" s="0">
-        <v>0.098623373038771583</v>
+        <v>0.030761094875371597</v>
       </c>
       <c r="G15" s="0">
-        <v>2.6164806530645572</v>
+        <v>3.1338443156560567</v>
       </c>
       <c r="H15" s="0">
         <v>1.5707963267948966</v>
       </c>
       <c r="I15" s="0">
-        <v>2.1845103513639877e-07</v>
+        <v>3.0803365020261157e-06</v>
       </c>
     </row>
   </sheetData>

</xml_diff>